<commit_message>
3주차 Rovoid 테스트케이스(TestCase)_1.2.0 업뎃
</commit_message>
<xml_diff>
--- a/QA/3주차 Rovoid 테스트케이스(TestCase)_1.2.0.xlsx
+++ b/QA/3주차 Rovoid 테스트케이스(TestCase)_1.2.0.xlsx
@@ -12,7 +12,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="UTrASsYVp3Uj1o/gIpkq0KDp8MeLN3VEydlbP/2/DZA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="0J9ug734Nxv6GJvkvWTBgjt8a3HA1TVL+TvZR4OonHc="/>
     </ext>
   </extLst>
 </workbook>
@@ -99,7 +99,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgmOcRqCzYC8bclPNTo2krFm45ZPw=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgZId8hfyqAYikr+K6+qJRmne/A5g=="/>
     </ext>
   </extLst>
 </comments>
@@ -476,7 +476,7 @@
 4. 'SELECT'를 클릭한다</t>
   </si>
   <si>
-    <t>스킬 1 OR 스킬 2이 선택될 것으로 예상된다</t>
+    <t>스킬 1 OR 스킬 2가 선택될 것으로 예상된다</t>
   </si>
   <si>
     <t>스킬이 선택됨</t>
@@ -650,7 +650,6 @@
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
     <font/>
     <font>
@@ -665,7 +664,6 @@
     <font>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -796,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="30">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -807,19 +805,13 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="2" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -828,51 +820,42 @@
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1302,1666 +1285,1666 @@
       <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="4" t="s">
+      <c r="K2" s="4"/>
+      <c r="L2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
     </row>
     <row r="3" ht="37.5" customHeight="1">
       <c r="A3" s="2">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="B3" s="9"/>
+      <c r="B3" s="7"/>
       <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="9"/>
-      <c r="G3" s="6" t="s">
+      <c r="F3" s="7"/>
+      <c r="G3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="11"/>
+      <c r="K3" s="8"/>
       <c r="L3" s="2" t="str">
         <f t="shared" ref="L3:L4" si="2">IF(B3="",L2,B3)</f>
         <v>게임실행</v>
       </c>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8"/>
-      <c r="Y3" s="8"/>
-      <c r="Z3" s="8"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
     </row>
     <row r="4" ht="37.5" customHeight="1">
       <c r="A4" s="2">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="12"/>
-      <c r="G4" s="10" t="s">
+      <c r="F4" s="9"/>
+      <c r="G4" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="11"/>
+      <c r="K4" s="8"/>
       <c r="L4" s="2" t="str">
         <f t="shared" si="2"/>
         <v>게임실행</v>
       </c>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="8"/>
-      <c r="W4" s="8"/>
-      <c r="X4" s="8"/>
-      <c r="Y4" s="8"/>
-      <c r="Z4" s="8"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
     </row>
     <row r="5" ht="37.5" customHeight="1">
       <c r="A5" s="2">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="8" t="s">
         <v>36</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="11"/>
-      <c r="L5" s="4" t="s">
+      <c r="K5" s="8"/>
+      <c r="L5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8"/>
-      <c r="Y5" s="8"/>
-      <c r="Z5" s="8"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6"/>
     </row>
     <row r="6">
       <c r="A6" s="2">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="10" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="10" t="s">
+      <c r="F6" s="7"/>
+      <c r="G6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="K6" s="11"/>
+      <c r="K6" s="8"/>
       <c r="L6" s="2" t="str">
         <f t="shared" ref="L6:L15" si="3">IF(B6="",L5,B6)</f>
         <v>인게임기능</v>
       </c>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="8"/>
-      <c r="W6" s="8"/>
-      <c r="X6" s="8"/>
-      <c r="Y6" s="8"/>
-      <c r="Z6" s="8"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6"/>
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="2">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="4" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="10" t="s">
+      <c r="F7" s="7"/>
+      <c r="G7" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="11"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
-      <c r="V7" s="8"/>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8"/>
-      <c r="Y7" s="8"/>
-      <c r="Z7" s="8"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
     </row>
     <row r="8" ht="37.5" customHeight="1">
       <c r="A8" s="2">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="10" t="s">
+      <c r="F8" s="7"/>
+      <c r="G8" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K8" s="11"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
-      <c r="V8" s="8"/>
-      <c r="W8" s="8"/>
-      <c r="X8" s="8"/>
-      <c r="Y8" s="8"/>
-      <c r="Z8" s="8"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
+      <c r="X8" s="6"/>
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6"/>
     </row>
     <row r="9" ht="37.5" customHeight="1">
       <c r="A9" s="2">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
       <c r="D9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="9"/>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="7"/>
+      <c r="G9" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="K9" s="11"/>
+      <c r="K9" s="8"/>
       <c r="L9" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="8"/>
-      <c r="S9" s="8"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="8"/>
-      <c r="V9" s="8"/>
-      <c r="W9" s="8"/>
-      <c r="X9" s="8"/>
-      <c r="Y9" s="8"/>
-      <c r="Z9" s="8"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6"/>
     </row>
     <row r="10" ht="37.5" customHeight="1">
       <c r="A10" s="2">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="10" t="s">
+      <c r="F10" s="7"/>
+      <c r="G10" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K10" s="11"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6"/>
+      <c r="Z10" s="6"/>
     </row>
     <row r="11" ht="37.5" customHeight="1">
       <c r="A11" s="2">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="10" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10" t="s">
+      <c r="F11" s="7"/>
+      <c r="G11" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K11" s="11"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="8"/>
-      <c r="S11" s="8"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="8"/>
-      <c r="W11" s="8"/>
-      <c r="X11" s="8"/>
-      <c r="Y11" s="8"/>
-      <c r="Z11" s="8"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
     </row>
     <row r="12" ht="37.5" customHeight="1">
       <c r="A12" s="2">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="10" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10" t="s">
+      <c r="F12" s="7"/>
+      <c r="G12" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="K12" s="11"/>
+      <c r="K12" s="8"/>
       <c r="L12" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8"/>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="8"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="6"/>
+      <c r="W12" s="6"/>
+      <c r="X12" s="6"/>
+      <c r="Y12" s="6"/>
+      <c r="Z12" s="6"/>
     </row>
     <row r="13" ht="37.5" customHeight="1">
       <c r="A13" s="2">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10" t="s">
+      <c r="F13" s="7"/>
+      <c r="G13" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="K13" s="11"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
-      <c r="W13" s="8"/>
-      <c r="X13" s="8"/>
-      <c r="Y13" s="8"/>
-      <c r="Z13" s="8"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
     </row>
     <row r="14" ht="37.5" customHeight="1">
       <c r="A14" s="2">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="14" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="14" t="s">
+      <c r="F14" s="7"/>
+      <c r="G14" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="15" t="s">
+      <c r="J14" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="12"/>
       <c r="L14" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M14" s="8"/>
-      <c r="N14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="8"/>
-      <c r="S14" s="8"/>
-      <c r="T14" s="8"/>
-      <c r="U14" s="8"/>
-      <c r="V14" s="8"/>
-      <c r="W14" s="8"/>
-      <c r="X14" s="8"/>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="8"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6"/>
     </row>
     <row r="15" ht="37.5" customHeight="1">
       <c r="A15" s="2">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="15" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="9"/>
-      <c r="G15" s="15" t="s">
+      <c r="F15" s="7"/>
+      <c r="G15" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="15" t="s">
+      <c r="J15" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="K15" s="16"/>
+      <c r="K15" s="12"/>
       <c r="L15" s="2" t="str">
         <f t="shared" si="3"/>
         <v>인게임기능</v>
       </c>
-      <c r="M15" s="8"/>
-      <c r="N15" s="8"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="8"/>
-      <c r="S15" s="8"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="8"/>
-      <c r="V15" s="8"/>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
-      <c r="Y15" s="8"/>
-      <c r="Z15" s="8"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="6"/>
+      <c r="Y15" s="6"/>
+      <c r="Z15" s="6"/>
     </row>
     <row r="16" ht="37.5" customHeight="1">
       <c r="A16" s="2">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="B16" s="9"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="F16" s="9"/>
-      <c r="G16" s="18" t="s">
+      <c r="F16" s="7"/>
+      <c r="G16" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J16" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="K16" s="11"/>
+      <c r="K16" s="8"/>
       <c r="L16" s="2" t="str">
         <f>IF(B14="",L13,B14)</f>
         <v>인게임기능</v>
       </c>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8"/>
-      <c r="S16" s="8"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="8"/>
-      <c r="V16" s="8"/>
-      <c r="W16" s="8"/>
-      <c r="X16" s="8"/>
-      <c r="Y16" s="8"/>
-      <c r="Z16" s="8"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
+      <c r="V16" s="6"/>
+      <c r="W16" s="6"/>
+      <c r="X16" s="6"/>
+      <c r="Y16" s="6"/>
+      <c r="Z16" s="6"/>
     </row>
     <row r="17" ht="37.5" customHeight="1">
       <c r="A17" s="2">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="17" t="s">
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="9"/>
-      <c r="G17" s="18" t="s">
+      <c r="F17" s="7"/>
+      <c r="G17" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="11"/>
+      <c r="K17" s="8"/>
       <c r="L17" s="2" t="str">
         <f t="shared" ref="L17:L20" si="4">IF(B15="",L16,B15)</f>
         <v>인게임기능</v>
       </c>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="8"/>
-      <c r="Z17" s="8"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
+      <c r="V17" s="6"/>
+      <c r="W17" s="6"/>
+      <c r="X17" s="6"/>
+      <c r="Y17" s="6"/>
+      <c r="Z17" s="6"/>
     </row>
     <row r="18" ht="37.5" customHeight="1">
       <c r="A18" s="2">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="17" t="s">
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="18" t="s">
+      <c r="F18" s="7"/>
+      <c r="G18" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="K18" s="11"/>
+      <c r="K18" s="8"/>
       <c r="L18" s="2" t="str">
         <f t="shared" si="4"/>
         <v>인게임기능</v>
       </c>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8"/>
-      <c r="S18" s="8"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="8"/>
-      <c r="V18" s="8"/>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
-      <c r="Y18" s="8"/>
-      <c r="Z18" s="8"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="6"/>
+      <c r="S18" s="6"/>
+      <c r="T18" s="6"/>
+      <c r="U18" s="6"/>
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
+      <c r="X18" s="6"/>
+      <c r="Y18" s="6"/>
+      <c r="Z18" s="6"/>
     </row>
     <row r="19" ht="37.5" customHeight="1">
       <c r="A19" s="2">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="17" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="18" t="s">
+      <c r="F19" s="7"/>
+      <c r="G19" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="J19" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="K19" s="11"/>
+      <c r="K19" s="8"/>
       <c r="L19" s="2" t="str">
         <f t="shared" si="4"/>
         <v>인게임기능</v>
       </c>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8"/>
-      <c r="S19" s="8"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="8"/>
-      <c r="V19" s="8"/>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
-      <c r="Y19" s="8"/>
-      <c r="Z19" s="8"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="6"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
+      <c r="X19" s="6"/>
+      <c r="Y19" s="6"/>
+      <c r="Z19" s="6"/>
     </row>
     <row r="20" ht="37.5" customHeight="1">
       <c r="A20" s="2">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="19" t="s">
+      <c r="B20" s="7"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="15" t="s">
+      <c r="F20" s="7"/>
+      <c r="G20" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="15" t="s">
+      <c r="J20" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="K20" s="16"/>
+      <c r="K20" s="12"/>
       <c r="L20" s="2" t="str">
         <f t="shared" si="4"/>
         <v>인게임기능</v>
       </c>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8"/>
-      <c r="S20" s="8"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="8"/>
-      <c r="V20" s="8"/>
-      <c r="W20" s="8"/>
-      <c r="X20" s="8"/>
-      <c r="Y20" s="8"/>
-      <c r="Z20" s="8"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="6"/>
+      <c r="S20" s="6"/>
+      <c r="T20" s="6"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="6"/>
+      <c r="W20" s="6"/>
+      <c r="X20" s="6"/>
+      <c r="Y20" s="6"/>
+      <c r="Z20" s="6"/>
     </row>
     <row r="21" ht="37.5" customHeight="1">
       <c r="A21" s="2">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="20" t="s">
+      <c r="B21" s="7"/>
+      <c r="C21" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="23" t="s">
+      <c r="F21" s="7"/>
+      <c r="G21" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="H21" s="22" t="s">
+      <c r="H21" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="I21" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="22" t="s">
+      <c r="J21" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="K21" s="11"/>
+      <c r="K21" s="8"/>
       <c r="L21" s="2" t="str">
         <f>IF(B18="",L19,B18)</f>
         <v>인게임기능</v>
       </c>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
-      <c r="Q21" s="8"/>
-      <c r="R21" s="8"/>
-      <c r="S21" s="8"/>
-      <c r="T21" s="8"/>
-      <c r="U21" s="8"/>
-      <c r="V21" s="8"/>
-      <c r="W21" s="8"/>
-      <c r="X21" s="8"/>
-      <c r="Y21" s="8"/>
-      <c r="Z21" s="8"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="6"/>
+      <c r="W21" s="6"/>
+      <c r="X21" s="6"/>
+      <c r="Y21" s="6"/>
+      <c r="Z21" s="6"/>
     </row>
     <row r="22" ht="37.5" customHeight="1">
       <c r="A22" s="2">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="20" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="F22" s="9"/>
-      <c r="G22" s="24" t="s">
+      <c r="F22" s="7"/>
+      <c r="G22" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="24" t="s">
+      <c r="H22" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I22" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="K22" s="11"/>
+      <c r="K22" s="8"/>
       <c r="L22" s="2" t="str">
         <f t="shared" ref="L22:L32" si="5">IF(B19="",L21,B19)</f>
         <v>인게임기능</v>
       </c>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="8"/>
-      <c r="S22" s="8"/>
-      <c r="T22" s="8"/>
-      <c r="U22" s="8"/>
-      <c r="V22" s="8"/>
-      <c r="W22" s="8"/>
-      <c r="X22" s="8"/>
-      <c r="Y22" s="8"/>
-      <c r="Z22" s="8"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6"/>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
+      <c r="V22" s="6"/>
+      <c r="W22" s="6"/>
+      <c r="X22" s="6"/>
+      <c r="Y22" s="6"/>
+      <c r="Z22" s="6"/>
     </row>
     <row r="23" ht="37.5" customHeight="1">
       <c r="A23" s="2">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="24" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="F23" s="9"/>
-      <c r="G23" s="24" t="s">
+      <c r="F23" s="7"/>
+      <c r="G23" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="H23" s="24" t="s">
+      <c r="H23" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="I23" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J23" s="22" t="s">
+      <c r="J23" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K23" s="11"/>
+      <c r="K23" s="8"/>
       <c r="L23" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
-      <c r="Q23" s="8"/>
-      <c r="R23" s="8"/>
-      <c r="S23" s="8"/>
-      <c r="T23" s="8"/>
-      <c r="U23" s="8"/>
-      <c r="V23" s="8"/>
-      <c r="W23" s="8"/>
-      <c r="X23" s="8"/>
-      <c r="Y23" s="8"/>
-      <c r="Z23" s="8"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6"/>
     </row>
     <row r="24" ht="37.5" customHeight="1">
       <c r="A24" s="2">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="24" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F24" s="9"/>
-      <c r="G24" s="24" t="s">
+      <c r="F24" s="7"/>
+      <c r="G24" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="H24" s="24" t="s">
+      <c r="H24" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J24" s="22" t="s">
+      <c r="J24" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K24" s="25"/>
+      <c r="K24" s="19"/>
       <c r="L24" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8"/>
-      <c r="S24" s="8"/>
-      <c r="T24" s="8"/>
-      <c r="U24" s="8"/>
-      <c r="V24" s="8"/>
-      <c r="W24" s="8"/>
-      <c r="X24" s="8"/>
-      <c r="Y24" s="8"/>
-      <c r="Z24" s="8"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
+      <c r="X24" s="6"/>
+      <c r="Y24" s="6"/>
+      <c r="Z24" s="6"/>
     </row>
     <row r="25" ht="37.5" customHeight="1">
       <c r="A25" s="2">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="24" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="F25" s="9"/>
-      <c r="G25" s="24" t="s">
+      <c r="F25" s="7"/>
+      <c r="G25" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="H25" s="24" t="s">
+      <c r="H25" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I25" s="7" t="s">
+      <c r="I25" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J25" s="22" t="s">
+      <c r="J25" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K25" s="25"/>
+      <c r="K25" s="19"/>
       <c r="L25" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
-      <c r="Q25" s="8"/>
-      <c r="R25" s="8"/>
-      <c r="S25" s="8"/>
-      <c r="T25" s="8"/>
-      <c r="U25" s="8"/>
-      <c r="V25" s="8"/>
-      <c r="W25" s="8"/>
-      <c r="X25" s="8"/>
-      <c r="Y25" s="8"/>
-      <c r="Z25" s="8"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
+      <c r="X25" s="6"/>
+      <c r="Y25" s="6"/>
+      <c r="Z25" s="6"/>
     </row>
     <row r="26" ht="37.5" customHeight="1">
       <c r="A26" s="2">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="20" t="s">
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="F26" s="9"/>
-      <c r="G26" s="24" t="s">
+      <c r="F26" s="7"/>
+      <c r="G26" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="H26" s="24" t="s">
+      <c r="H26" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J26" s="22" t="s">
+      <c r="J26" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K26" s="25"/>
+      <c r="K26" s="19"/>
       <c r="L26" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="8"/>
-      <c r="S26" s="8"/>
-      <c r="T26" s="8"/>
-      <c r="U26" s="8"/>
-      <c r="V26" s="8"/>
-      <c r="W26" s="8"/>
-      <c r="X26" s="8"/>
-      <c r="Y26" s="8"/>
-      <c r="Z26" s="8"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
+      <c r="X26" s="6"/>
+      <c r="Y26" s="6"/>
+      <c r="Z26" s="6"/>
     </row>
     <row r="27" ht="37.5" customHeight="1">
       <c r="A27" s="2">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="24" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="24" t="s">
+      <c r="F27" s="7"/>
+      <c r="G27" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="H27" s="24" t="s">
+      <c r="H27" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J27" s="22" t="s">
+      <c r="J27" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K27" s="23"/>
+      <c r="K27" s="17"/>
       <c r="L27" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
-      <c r="Q27" s="8"/>
-      <c r="R27" s="8"/>
-      <c r="S27" s="8"/>
-      <c r="T27" s="8"/>
-      <c r="U27" s="8"/>
-      <c r="V27" s="8"/>
-      <c r="W27" s="8"/>
-      <c r="X27" s="8"/>
-      <c r="Y27" s="8"/>
-      <c r="Z27" s="8"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="6"/>
+      <c r="Y27" s="6"/>
+      <c r="Z27" s="6"/>
     </row>
     <row r="28" ht="37.5" customHeight="1">
       <c r="A28" s="2">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="24" t="s">
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="F28" s="9"/>
-      <c r="G28" s="24" t="s">
+      <c r="F28" s="7"/>
+      <c r="G28" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H28" s="24" t="s">
+      <c r="H28" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="I28" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J28" s="22" t="s">
+      <c r="J28" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K28" s="25"/>
+      <c r="K28" s="19"/>
       <c r="L28" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
-      <c r="Q28" s="8"/>
-      <c r="R28" s="8"/>
-      <c r="S28" s="8"/>
-      <c r="T28" s="8"/>
-      <c r="U28" s="8"/>
-      <c r="V28" s="8"/>
-      <c r="W28" s="8"/>
-      <c r="X28" s="8"/>
-      <c r="Y28" s="8"/>
-      <c r="Z28" s="8"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
+      <c r="X28" s="6"/>
+      <c r="Y28" s="6"/>
+      <c r="Z28" s="6"/>
     </row>
     <row r="29" ht="37.5" customHeight="1">
       <c r="A29" s="2">
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="24" t="s">
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="9"/>
-      <c r="G29" s="24" t="s">
+      <c r="F29" s="7"/>
+      <c r="G29" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="24" t="s">
+      <c r="H29" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I29" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J29" s="22" t="s">
+      <c r="J29" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K29" s="25"/>
+      <c r="K29" s="19"/>
       <c r="L29" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="8"/>
-      <c r="S29" s="8"/>
-      <c r="T29" s="8"/>
-      <c r="U29" s="8"/>
-      <c r="V29" s="8"/>
-      <c r="W29" s="8"/>
-      <c r="X29" s="8"/>
-      <c r="Y29" s="8"/>
-      <c r="Z29" s="8"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6"/>
+      <c r="T29" s="6"/>
+      <c r="U29" s="6"/>
+      <c r="V29" s="6"/>
+      <c r="W29" s="6"/>
+      <c r="X29" s="6"/>
+      <c r="Y29" s="6"/>
+      <c r="Z29" s="6"/>
     </row>
     <row r="30" ht="37.5" customHeight="1">
       <c r="A30" s="2">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="19" t="s">
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="15" t="s">
+      <c r="F30" s="7"/>
+      <c r="G30" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J30" s="22" t="s">
+      <c r="J30" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K30" s="25"/>
+      <c r="K30" s="19"/>
       <c r="L30" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8"/>
-      <c r="S30" s="8"/>
-      <c r="T30" s="8"/>
-      <c r="U30" s="8"/>
-      <c r="V30" s="8"/>
-      <c r="W30" s="8"/>
-      <c r="X30" s="8"/>
-      <c r="Y30" s="8"/>
-      <c r="Z30" s="8"/>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
+      <c r="R30" s="6"/>
+      <c r="S30" s="6"/>
+      <c r="T30" s="6"/>
+      <c r="U30" s="6"/>
+      <c r="V30" s="6"/>
+      <c r="W30" s="6"/>
+      <c r="X30" s="6"/>
+      <c r="Y30" s="6"/>
+      <c r="Z30" s="6"/>
     </row>
     <row r="31" ht="37.5" customHeight="1">
       <c r="A31" s="2">
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="21" t="s">
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="F31" s="9"/>
-      <c r="G31" s="15" t="s">
+      <c r="F31" s="7"/>
+      <c r="G31" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I31" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J31" s="22" t="s">
+      <c r="J31" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K31" s="25"/>
+      <c r="K31" s="19"/>
       <c r="L31" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8"/>
-      <c r="S31" s="8"/>
-      <c r="T31" s="8"/>
-      <c r="U31" s="8"/>
-      <c r="V31" s="8"/>
-      <c r="W31" s="8"/>
-      <c r="X31" s="8"/>
-      <c r="Y31" s="8"/>
-      <c r="Z31" s="8"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
+      <c r="W31" s="6"/>
+      <c r="X31" s="6"/>
+      <c r="Y31" s="6"/>
+      <c r="Z31" s="6"/>
     </row>
     <row r="32" ht="37.5" customHeight="1">
       <c r="A32" s="2">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="21" t="s">
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="15" t="s">
+      <c r="F32" s="9"/>
+      <c r="G32" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="H32" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="I32" s="7" t="s">
+      <c r="I32" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J32" s="22" t="s">
+      <c r="J32" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K32" s="25"/>
+      <c r="K32" s="19"/>
       <c r="L32" s="2" t="str">
         <f t="shared" si="5"/>
         <v>인게임기능</v>
       </c>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8"/>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8"/>
-      <c r="S32" s="8"/>
-      <c r="T32" s="8"/>
-      <c r="U32" s="8"/>
-      <c r="V32" s="8"/>
-      <c r="W32" s="8"/>
-      <c r="X32" s="8"/>
-      <c r="Y32" s="8"/>
-      <c r="Z32" s="8"/>
+      <c r="M32" s="6"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+      <c r="T32" s="6"/>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+      <c r="W32" s="6"/>
+      <c r="X32" s="6"/>
+      <c r="Y32" s="6"/>
+      <c r="Z32" s="6"/>
     </row>
     <row r="33" ht="37.5" customHeight="1">
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
-      <c r="Q33" s="8"/>
-      <c r="R33" s="8"/>
-      <c r="S33" s="8"/>
-      <c r="T33" s="8"/>
-      <c r="U33" s="8"/>
-      <c r="V33" s="8"/>
-      <c r="W33" s="8"/>
-      <c r="X33" s="8"/>
-      <c r="Y33" s="8"/>
-      <c r="Z33" s="8"/>
+      <c r="M33" s="20"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+      <c r="R33" s="6"/>
+      <c r="S33" s="6"/>
+      <c r="T33" s="6"/>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6"/>
+      <c r="W33" s="6"/>
+      <c r="X33" s="6"/>
+      <c r="Y33" s="6"/>
+      <c r="Z33" s="6"/>
     </row>
     <row r="34" ht="37.5" customHeight="1">
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="8"/>
-      <c r="S34" s="8"/>
-      <c r="T34" s="8"/>
-      <c r="U34" s="8"/>
-      <c r="V34" s="8"/>
-      <c r="W34" s="8"/>
-      <c r="X34" s="8"/>
-      <c r="Y34" s="8"/>
-      <c r="Z34" s="8"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
+      <c r="R34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6"/>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6"/>
+      <c r="W34" s="6"/>
+      <c r="X34" s="6"/>
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="6"/>
     </row>
     <row r="35" ht="37.5" customHeight="1">
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="8"/>
-      <c r="W35" s="8"/>
-      <c r="X35" s="8"/>
-      <c r="Y35" s="8"/>
-      <c r="Z35" s="8"/>
+      <c r="M35" s="6"/>
+      <c r="N35" s="6"/>
+      <c r="O35" s="6"/>
+      <c r="P35" s="6"/>
+      <c r="Q35" s="6"/>
+      <c r="R35" s="6"/>
+      <c r="S35" s="6"/>
+      <c r="T35" s="6"/>
+      <c r="U35" s="6"/>
+      <c r="V35" s="6"/>
+      <c r="W35" s="6"/>
+      <c r="X35" s="6"/>
+      <c r="Y35" s="6"/>
+      <c r="Z35" s="6"/>
     </row>
     <row r="36" ht="37.5" customHeight="1">
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="8"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="8"/>
-      <c r="W36" s="8"/>
-      <c r="X36" s="8"/>
-      <c r="Y36" s="8"/>
-      <c r="Z36" s="8"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6"/>
+      <c r="R36" s="6"/>
+      <c r="S36" s="6"/>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+      <c r="W36" s="6"/>
+      <c r="X36" s="6"/>
+      <c r="Y36" s="6"/>
+      <c r="Z36" s="6"/>
     </row>
     <row r="37" ht="37.5" customHeight="1">
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
-      <c r="Q37" s="8"/>
-      <c r="R37" s="8"/>
-      <c r="S37" s="8"/>
-      <c r="T37" s="8"/>
-      <c r="U37" s="8"/>
-      <c r="V37" s="8"/>
-      <c r="W37" s="8"/>
-      <c r="X37" s="8"/>
-      <c r="Y37" s="8"/>
-      <c r="Z37" s="8"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6"/>
+      <c r="R37" s="6"/>
+      <c r="S37" s="6"/>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
+      <c r="X37" s="6"/>
+      <c r="Y37" s="6"/>
+      <c r="Z37" s="6"/>
     </row>
     <row r="38" ht="37.5" customHeight="1">
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
-      <c r="S38" s="8"/>
-      <c r="T38" s="8"/>
-      <c r="U38" s="8"/>
-      <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
-      <c r="X38" s="8"/>
-      <c r="Y38" s="8"/>
-      <c r="Z38" s="8"/>
+      <c r="M38" s="6"/>
+      <c r="N38" s="6"/>
+      <c r="O38" s="6"/>
+      <c r="P38" s="6"/>
+      <c r="Q38" s="6"/>
+      <c r="R38" s="6"/>
+      <c r="S38" s="6"/>
+      <c r="T38" s="6"/>
+      <c r="U38" s="6"/>
+      <c r="V38" s="6"/>
+      <c r="W38" s="6"/>
+      <c r="X38" s="6"/>
+      <c r="Y38" s="6"/>
+      <c r="Z38" s="6"/>
     </row>
     <row r="39" ht="37.5" customHeight="1">
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
-      <c r="S39" s="8"/>
-      <c r="T39" s="8"/>
-      <c r="U39" s="8"/>
-      <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
-      <c r="X39" s="8"/>
-      <c r="Y39" s="8"/>
-      <c r="Z39" s="8"/>
+      <c r="M39" s="6"/>
+      <c r="N39" s="6"/>
+      <c r="O39" s="6"/>
+      <c r="P39" s="6"/>
+      <c r="Q39" s="6"/>
+      <c r="R39" s="6"/>
+      <c r="S39" s="6"/>
+      <c r="T39" s="6"/>
+      <c r="U39" s="6"/>
+      <c r="V39" s="6"/>
+      <c r="W39" s="6"/>
+      <c r="X39" s="6"/>
+      <c r="Y39" s="6"/>
+      <c r="Z39" s="6"/>
     </row>
     <row r="40" ht="37.5" customHeight="1">
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
-      <c r="P40" s="8"/>
-      <c r="Q40" s="8"/>
-      <c r="R40" s="8"/>
-      <c r="S40" s="8"/>
-      <c r="T40" s="8"/>
-      <c r="U40" s="8"/>
-      <c r="V40" s="8"/>
-      <c r="W40" s="8"/>
-      <c r="X40" s="8"/>
-      <c r="Y40" s="8"/>
-      <c r="Z40" s="8"/>
+      <c r="M40" s="6"/>
+      <c r="N40" s="6"/>
+      <c r="O40" s="6"/>
+      <c r="P40" s="6"/>
+      <c r="Q40" s="6"/>
+      <c r="R40" s="6"/>
+      <c r="S40" s="6"/>
+      <c r="T40" s="6"/>
+      <c r="U40" s="6"/>
+      <c r="V40" s="6"/>
+      <c r="W40" s="6"/>
+      <c r="X40" s="6"/>
+      <c r="Y40" s="6"/>
+      <c r="Z40" s="6"/>
     </row>
     <row r="41" ht="37.5" customHeight="1">
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
-      <c r="P41" s="8"/>
-      <c r="Q41" s="8"/>
-      <c r="R41" s="8"/>
-      <c r="S41" s="8"/>
-      <c r="T41" s="8"/>
-      <c r="U41" s="8"/>
-      <c r="V41" s="8"/>
-      <c r="W41" s="8"/>
-      <c r="X41" s="8"/>
-      <c r="Y41" s="8"/>
-      <c r="Z41" s="8"/>
+      <c r="M41" s="6"/>
+      <c r="N41" s="6"/>
+      <c r="O41" s="6"/>
+      <c r="P41" s="6"/>
+      <c r="Q41" s="6"/>
+      <c r="R41" s="6"/>
+      <c r="S41" s="6"/>
+      <c r="T41" s="6"/>
+      <c r="U41" s="6"/>
+      <c r="V41" s="6"/>
+      <c r="W41" s="6"/>
+      <c r="X41" s="6"/>
+      <c r="Y41" s="6"/>
+      <c r="Z41" s="6"/>
     </row>
     <row r="42" ht="37.5" customHeight="1">
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
-      <c r="P42" s="8"/>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
-      <c r="S42" s="8"/>
-      <c r="T42" s="8"/>
-      <c r="U42" s="8"/>
-      <c r="V42" s="8"/>
-      <c r="W42" s="8"/>
-      <c r="X42" s="8"/>
-      <c r="Y42" s="8"/>
-      <c r="Z42" s="8"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="6"/>
+      <c r="Q42" s="6"/>
+      <c r="R42" s="6"/>
+      <c r="S42" s="6"/>
+      <c r="T42" s="6"/>
+      <c r="U42" s="6"/>
+      <c r="V42" s="6"/>
+      <c r="W42" s="6"/>
+      <c r="X42" s="6"/>
+      <c r="Y42" s="6"/>
+      <c r="Z42" s="6"/>
     </row>
     <row r="43" ht="37.5" customHeight="1">
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
-      <c r="P43" s="8"/>
-      <c r="Q43" s="8"/>
-      <c r="R43" s="8"/>
-      <c r="S43" s="8"/>
-      <c r="T43" s="8"/>
-      <c r="U43" s="8"/>
-      <c r="V43" s="8"/>
-      <c r="W43" s="8"/>
-      <c r="X43" s="8"/>
-      <c r="Y43" s="8"/>
-      <c r="Z43" s="8"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+      <c r="S43" s="6"/>
+      <c r="T43" s="6"/>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
+      <c r="X43" s="6"/>
+      <c r="Y43" s="6"/>
+      <c r="Z43" s="6"/>
     </row>
     <row r="44" ht="37.5" customHeight="1">
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
-      <c r="P44" s="8"/>
-      <c r="Q44" s="8"/>
-      <c r="R44" s="8"/>
-      <c r="S44" s="8"/>
-      <c r="T44" s="8"/>
-      <c r="U44" s="8"/>
-      <c r="V44" s="8"/>
-      <c r="W44" s="8"/>
-      <c r="X44" s="8"/>
-      <c r="Y44" s="8"/>
-      <c r="Z44" s="8"/>
+      <c r="M44" s="6"/>
+      <c r="N44" s="6"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
+      <c r="Q44" s="6"/>
+      <c r="R44" s="6"/>
+      <c r="S44" s="6"/>
+      <c r="T44" s="6"/>
+      <c r="U44" s="6"/>
+      <c r="V44" s="6"/>
+      <c r="W44" s="6"/>
+      <c r="X44" s="6"/>
+      <c r="Y44" s="6"/>
+      <c r="Z44" s="6"/>
     </row>
     <row r="45" ht="37.5" customHeight="1">
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
-      <c r="P45" s="8"/>
-      <c r="Q45" s="8"/>
-      <c r="R45" s="8"/>
-      <c r="S45" s="8"/>
-      <c r="T45" s="8"/>
-      <c r="U45" s="8"/>
-      <c r="V45" s="8"/>
-      <c r="W45" s="8"/>
-      <c r="X45" s="8"/>
-      <c r="Y45" s="8"/>
-      <c r="Z45" s="8"/>
+      <c r="M45" s="6"/>
+      <c r="N45" s="6"/>
+      <c r="O45" s="6"/>
+      <c r="P45" s="6"/>
+      <c r="Q45" s="6"/>
+      <c r="R45" s="6"/>
+      <c r="S45" s="6"/>
+      <c r="T45" s="6"/>
+      <c r="U45" s="6"/>
+      <c r="V45" s="6"/>
+      <c r="W45" s="6"/>
+      <c r="X45" s="6"/>
+      <c r="Y45" s="6"/>
+      <c r="Z45" s="6"/>
     </row>
     <row r="46">
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
-      <c r="Q46" s="8"/>
-      <c r="R46" s="8"/>
-      <c r="S46" s="8"/>
-      <c r="T46" s="8"/>
-      <c r="U46" s="8"/>
-      <c r="V46" s="8"/>
-      <c r="W46" s="8"/>
-      <c r="X46" s="8"/>
-      <c r="Y46" s="8"/>
-      <c r="Z46" s="8"/>
+      <c r="M46" s="6"/>
+      <c r="N46" s="6"/>
+      <c r="O46" s="6"/>
+      <c r="P46" s="6"/>
+      <c r="Q46" s="6"/>
+      <c r="R46" s="6"/>
+      <c r="S46" s="6"/>
+      <c r="T46" s="6"/>
+      <c r="U46" s="6"/>
+      <c r="V46" s="6"/>
+      <c r="W46" s="6"/>
+      <c r="X46" s="6"/>
+      <c r="Y46" s="6"/>
+      <c r="Z46" s="6"/>
     </row>
     <row r="47" ht="37.5" customHeight="1">
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-      <c r="P47" s="8"/>
-      <c r="Q47" s="8"/>
-      <c r="R47" s="8"/>
-      <c r="S47" s="8"/>
-      <c r="T47" s="8"/>
-      <c r="U47" s="8"/>
-      <c r="V47" s="8"/>
-      <c r="W47" s="8"/>
-      <c r="X47" s="8"/>
-      <c r="Y47" s="8"/>
-      <c r="Z47" s="8"/>
+      <c r="M47" s="6"/>
+      <c r="N47" s="6"/>
+      <c r="O47" s="6"/>
+      <c r="P47" s="6"/>
+      <c r="Q47" s="6"/>
+      <c r="R47" s="6"/>
+      <c r="S47" s="6"/>
+      <c r="T47" s="6"/>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+      <c r="W47" s="6"/>
+      <c r="X47" s="6"/>
+      <c r="Y47" s="6"/>
+      <c r="Z47" s="6"/>
     </row>
     <row r="48" ht="37.5" customHeight="1">
-      <c r="M48" s="8"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
-      <c r="P48" s="8"/>
-      <c r="Q48" s="8"/>
-      <c r="R48" s="8"/>
-      <c r="S48" s="8"/>
-      <c r="T48" s="8"/>
-      <c r="U48" s="8"/>
-      <c r="V48" s="8"/>
-      <c r="W48" s="8"/>
-      <c r="X48" s="8"/>
-      <c r="Y48" s="8"/>
-      <c r="Z48" s="8"/>
+      <c r="M48" s="6"/>
+      <c r="N48" s="6"/>
+      <c r="O48" s="6"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="6"/>
+      <c r="R48" s="6"/>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
+      <c r="X48" s="6"/>
+      <c r="Y48" s="6"/>
+      <c r="Z48" s="6"/>
     </row>
     <row r="49" ht="37.5" customHeight="1"/>
     <row r="50" ht="37.5" customHeight="1"/>
@@ -3917,18 +3900,18 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C5:C15"/>
+    <mergeCell ref="C16:C20"/>
+    <mergeCell ref="D9:D15"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="B2:B4"/>
     <mergeCell ref="F2:F4"/>
-    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B5:B32"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F5:F32"/>
+    <mergeCell ref="C21:C32"/>
     <mergeCell ref="D26:D29"/>
-    <mergeCell ref="C16:C20"/>
-    <mergeCell ref="C21:C32"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="C5:C15"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D9:D15"/>
-    <mergeCell ref="B5:B32"/>
-    <mergeCell ref="F5:F32"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:G1">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
@@ -4041,11 +4024,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I32">
+      <formula1>"Pass,Fail,Block,N/A,N/T"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L32">
       <formula1>"게임실행,메뉴기능,인게임기능"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I32">
-      <formula1>"Pass,Fail,Block,N/A,N/T"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions/>
@@ -4073,234 +4056,234 @@
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="21" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="I2" s="27" t="s">
+      <c r="I2" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="J2" s="22" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="29">
+      <c r="B3" s="24">
         <f>COUNTIF(TestCase!L:L,A3)</f>
         <v>3</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="25">
         <f t="shared" ref="C3:C5" si="1">IFERROR(B3/$B$6,0)</f>
         <v>0.09677419355</v>
       </c>
-      <c r="D3" s="29">
+      <c r="D3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;D$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>3</v>
       </c>
-      <c r="E3" s="29">
+      <c r="E3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;E$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>0</v>
       </c>
-      <c r="F3" s="29">
+      <c r="F3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;F$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>0</v>
       </c>
-      <c r="G3" s="29">
+      <c r="G3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;G$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="29">
+      <c r="H3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;H$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>0</v>
       </c>
-      <c r="I3" s="29">
+      <c r="I3" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;I$2&amp;"*",TestCase!$L:$L,$A3)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="31">
+      <c r="J3" s="26">
         <f t="shared" ref="J3:J5" si="2">I3/B3</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="24">
         <f>COUNTIF(TestCase!L:L,A4)</f>
         <v>0</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="25">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D4" s="29">
+      <c r="D4" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;D$2&amp;"*",TestCase!$L:$L,$A4)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;E$2&amp;"*",TestCase!$L:$L,$A4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="29">
+      <c r="F4" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;F$2&amp;"*",TestCase!$L:$L,$A4)</f>
         <v>0</v>
       </c>
-      <c r="G4" s="29">
+      <c r="G4" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;G$2&amp;"*",TestCase!$L:$L,$A4)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="29">
+      <c r="H4" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;H$2&amp;"*",TestCase!$L:$L,$A4)</f>
         <v>0</v>
       </c>
-      <c r="I4" s="32">
+      <c r="I4" s="27">
         <f t="shared" ref="I4:I5" si="3">SUM(D4:H4)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="31" t="str">
+      <c r="J4" s="26" t="str">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="24">
         <f>COUNTIF(TestCase!L:L,A5)</f>
         <v>28</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="25">
         <f t="shared" si="1"/>
         <v>0.9032258065</v>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;D$2&amp;"*",TestCase!$L:$L,$A5)</f>
         <v>15</v>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;E$2&amp;"*",TestCase!$L:$L,$A5)</f>
         <v>13</v>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;F$2&amp;"*",TestCase!$L:$L,$A5)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;G$2&amp;"*",TestCase!$L:$L,$A5)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="29">
+      <c r="H5" s="24">
         <f>COUNTIFS(TestCase!$I:$I,"*"&amp;H$2&amp;"*",TestCase!$L:$L,$A5)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="32">
+      <c r="I5" s="27">
         <f t="shared" si="3"/>
         <v>28</v>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="26">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="28">
         <f t="shared" ref="B6:I6" si="4">SUM(B3:B5)</f>
         <v>31</v>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="29">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="27">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="27">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="27">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="27">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="27">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I6" s="32">
+      <c r="I6" s="27">
         <f t="shared" si="4"/>
         <v>28</v>
       </c>
-      <c r="J6" s="32"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="31">
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="26">
         <f t="shared" ref="D7:I7" si="5">D6/$B6</f>
         <v>0.5806451613</v>
       </c>
-      <c r="E7" s="31">
+      <c r="E7" s="26">
         <f t="shared" si="5"/>
         <v>0.4193548387</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="26">
         <f t="shared" si="5"/>
         <v>0.9032258065</v>
       </c>
-      <c r="J7" s="32"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" ht="12.75" customHeight="1"/>
     <row r="9" ht="12.75" customHeight="1"/>

</xml_diff>